<commit_message>
fix: clean up .idea and pycache from git, update .gitignore, regenerate plots and reports
</commit_message>
<xml_diff>
--- a/lab2/supermarket_simulation.xlsx
+++ b/lab2/supermarket_simulation.xlsx
@@ -21681,7 +21681,7 @@
         <v>0.883</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -21709,7 +21709,7 @@
         <v>2.612</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0.662</v>
@@ -21765,7 +21765,7 @@
         <v>4.278</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
         <v>0.404</v>
@@ -21779,7 +21779,7 @@
         <v>5.283</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
         <v>0.518</v>
@@ -21793,7 +21793,7 @@
         <v>5.747</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
         <v>0.637</v>
@@ -21835,7 +21835,7 @@
         <v>7.351</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0.716</v>
@@ -21849,7 +21849,7 @@
         <v>8.021000000000001</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
         <v>0.657</v>
@@ -21863,7 +21863,7 @@
         <v>8.41</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0.672</v>
@@ -21877,7 +21877,7 @@
         <v>8.872</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
         <v>0.637</v>
@@ -21947,7 +21947,7 @@
         <v>9.971</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0.677</v>
@@ -21961,7 +21961,7 @@
         <v>11.766</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
         <v>0.574</v>
@@ -21989,7 +21989,7 @@
         <v>12.076</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0.585</v>
@@ -22017,7 +22017,7 @@
         <v>13.412</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
         <v>0.527</v>
@@ -22031,7 +22031,7 @@
         <v>13.931</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0.544</v>
@@ -22045,7 +22045,7 @@
         <v>14.254</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>0.532</v>
@@ -22073,7 +22073,7 @@
         <v>14.929</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0.553</v>
@@ -22087,7 +22087,7 @@
         <v>15.757</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
         <v>0.524</v>
@@ -22101,7 +22101,7 @@
         <v>15.842</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
         <v>0.527</v>
@@ -22129,7 +22129,7 @@
         <v>16.372</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
         <v>0.574</v>
@@ -22143,7 +22143,7 @@
         <v>16.428</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
         <v>0.583</v>
@@ -22157,7 +22157,7 @@
         <v>16.629</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
         <v>0.624</v>
@@ -22171,7 +22171,7 @@
         <v>17.169</v>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
         <v>0.699</v>
@@ -22185,7 +22185,7 @@
         <v>17.276</v>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
         <v>0.719</v>
@@ -22199,7 +22199,7 @@
         <v>17.305</v>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
         <v>0.723</v>
@@ -22213,7 +22213,7 @@
         <v>18.724</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
         <v>0.971</v>
@@ -22241,7 +22241,7 @@
         <v>18.908</v>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
         <v>0.991</v>
@@ -22255,7 +22255,7 @@
         <v>19.03</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
         <v>0.998</v>
@@ -22269,7 +22269,7 @@
         <v>19.051</v>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
         <v>1</v>
@@ -22283,7 +22283,7 @@
         <v>19.63</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
         <v>1.029</v>
@@ -22297,7 +22297,7 @@
         <v>20.299</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
         <v>1.094</v>
@@ -22339,7 +22339,7 @@
         <v>21.139</v>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
         <v>1.21</v>
@@ -22367,7 +22367,7 @@
         <v>21.919</v>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>1.273</v>
@@ -22409,7 +22409,7 @@
         <v>23.151</v>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D55" t="n">
         <v>1.418</v>
@@ -22437,7 +22437,7 @@
         <v>23.261</v>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D57" t="n">
         <v>1.435</v>
@@ -22451,7 +22451,7 @@
         <v>23.39</v>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D58" t="n">
         <v>1.45</v>
@@ -22493,7 +22493,7 @@
         <v>24.018</v>
       </c>
       <c r="C61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D61" t="n">
         <v>1.542</v>
@@ -22521,7 +22521,7 @@
         <v>24.378</v>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D63" t="n">
         <v>1.608</v>
@@ -22535,7 +22535,7 @@
         <v>24.683</v>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D64" t="n">
         <v>1.675</v>
@@ -22549,7 +22549,7 @@
         <v>25.205</v>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D65" t="n">
         <v>1.764</v>
@@ -22563,7 +22563,7 @@
         <v>25.372</v>
       </c>
       <c r="C66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D66" t="n">
         <v>1.786</v>
@@ -22577,7 +22577,7 @@
         <v>25.635</v>
       </c>
       <c r="C67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D67" t="n">
         <v>1.829</v>
@@ -22591,7 +22591,7 @@
         <v>26.059</v>
       </c>
       <c r="C68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
         <v>1.88</v>
@@ -22605,7 +22605,7 @@
         <v>26.522</v>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D69" t="n">
         <v>1.917</v>
@@ -22619,7 +22619,7 @@
         <v>27.003</v>
       </c>
       <c r="C70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
         <v>1.972</v>
@@ -22647,7 +22647,7 @@
         <v>27.599</v>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
         <v>2.016</v>
@@ -22675,7 +22675,7 @@
         <v>28.153</v>
       </c>
       <c r="C74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D74" t="n">
         <v>2.036</v>
@@ -22717,7 +22717,7 @@
         <v>28.768</v>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D77" t="n">
         <v>2.078</v>
@@ -22745,7 +22745,7 @@
         <v>28.966</v>
       </c>
       <c r="C79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D79" t="n">
         <v>2.097</v>
@@ -22759,7 +22759,7 @@
         <v>29.02</v>
       </c>
       <c r="C80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D80" t="n">
         <v>2.105</v>
@@ -22773,7 +22773,7 @@
         <v>29.244</v>
       </c>
       <c r="C81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D81" t="n">
         <v>2.142</v>
@@ -22787,7 +22787,7 @@
         <v>29.972</v>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D82" t="n">
         <v>2.236</v>
@@ -22801,7 +22801,7 @@
         <v>30.37</v>
       </c>
       <c r="C83" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D83" t="n">
         <v>2.298</v>
@@ -22829,7 +22829,7 @@
         <v>30.552</v>
       </c>
       <c r="C85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D85" t="n">
         <v>2.332</v>
@@ -22843,7 +22843,7 @@
         <v>30.822</v>
       </c>
       <c r="C86" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D86" t="n">
         <v>2.373</v>
@@ -22885,7 +22885,7 @@
         <v>32.461</v>
       </c>
       <c r="C89" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D89" t="n">
         <v>2.657</v>
@@ -22913,7 +22913,7 @@
         <v>32.966</v>
       </c>
       <c r="C91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D91" t="n">
         <v>2.755</v>
@@ -22941,7 +22941,7 @@
         <v>33.465</v>
       </c>
       <c r="C93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D93" t="n">
         <v>2.833</v>
@@ -23025,7 +23025,7 @@
         <v>35.471</v>
       </c>
       <c r="C99" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D99" t="n">
         <v>3.182</v>
@@ -23067,7 +23067,7 @@
         <v>36.394</v>
       </c>
       <c r="C102" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D102" t="n">
         <v>3.304</v>
@@ -23081,7 +23081,7 @@
         <v>36.486</v>
       </c>
       <c r="C103" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D103" t="n">
         <v>3.313</v>
@@ -23123,7 +23123,7 @@
         <v>37.836</v>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D106" t="n">
         <v>3.48</v>
@@ -23151,7 +23151,7 @@
         <v>37.995</v>
       </c>
       <c r="C108" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D108" t="n">
         <v>3.495</v>
@@ -23179,7 +23179,7 @@
         <v>38.962</v>
       </c>
       <c r="C110" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D110" t="n">
         <v>3.557</v>
@@ -23235,7 +23235,7 @@
         <v>40.497</v>
       </c>
       <c r="C114" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D114" t="n">
         <v>3.688</v>
@@ -23249,7 +23249,7 @@
         <v>40.729</v>
       </c>
       <c r="C115" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D115" t="n">
         <v>3.701</v>
@@ -23263,7 +23263,7 @@
         <v>41.179</v>
       </c>
       <c r="C116" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D116" t="n">
         <v>3.737</v>
@@ -23291,7 +23291,7 @@
         <v>41.469</v>
       </c>
       <c r="C118" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D118" t="n">
         <v>3.767</v>
@@ -23305,7 +23305,7 @@
         <v>41.546</v>
       </c>
       <c r="C119" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D119" t="n">
         <v>3.773</v>
@@ -23319,7 +23319,7 @@
         <v>42.285</v>
       </c>
       <c r="C120" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D120" t="n">
         <v>3.847</v>
@@ -23333,7 +23333,7 @@
         <v>42.707</v>
       </c>
       <c r="C121" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D121" t="n">
         <v>3.878</v>
@@ -23361,7 +23361,7 @@
         <v>42.977</v>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D123" t="n">
         <v>3.904</v>
@@ -23389,7 +23389,7 @@
         <v>44.434</v>
       </c>
       <c r="C125" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D125" t="n">
         <v>4.071</v>
@@ -23459,7 +23459,7 @@
         <v>45.497</v>
       </c>
       <c r="C130" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D130" t="n">
         <v>4.163</v>
@@ -23473,7 +23473,7 @@
         <v>45.696</v>
       </c>
       <c r="C131" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D131" t="n">
         <v>4.184</v>
@@ -23487,7 +23487,7 @@
         <v>45.94</v>
       </c>
       <c r="C132" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D132" t="n">
         <v>4.204</v>
@@ -23515,7 +23515,7 @@
         <v>46.184</v>
       </c>
       <c r="C134" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D134" t="n">
         <v>4.229</v>
@@ -23529,7 +23529,7 @@
         <v>46.233</v>
       </c>
       <c r="C135" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D135" t="n">
         <v>4.235</v>
@@ -23543,7 +23543,7 @@
         <v>46.44</v>
       </c>
       <c r="C136" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D136" t="n">
         <v>4.266</v>
@@ -23557,7 +23557,7 @@
         <v>46.734</v>
       </c>
       <c r="C137" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D137" t="n">
         <v>4.314</v>
@@ -23571,7 +23571,7 @@
         <v>46.8</v>
       </c>
       <c r="C138" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D138" t="n">
         <v>4.326</v>
@@ -23613,7 +23613,7 @@
         <v>47.185</v>
       </c>
       <c r="C141" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D141" t="n">
         <v>4.405</v>
@@ -23641,7 +23641,7 @@
         <v>48.382</v>
       </c>
       <c r="C143" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D143" t="n">
         <v>4.618</v>
@@ -23655,7 +23655,7 @@
         <v>48.704</v>
       </c>
       <c r="C144" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D144" t="n">
         <v>4.68</v>
@@ -23683,7 +23683,7 @@
         <v>48.941</v>
       </c>
       <c r="C146" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D146" t="n">
         <v>4.73</v>
@@ -23697,7 +23697,7 @@
         <v>49.154</v>
       </c>
       <c r="C147" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D147" t="n">
         <v>4.77</v>
@@ -23739,7 +23739,7 @@
         <v>50.133</v>
       </c>
       <c r="C150" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D150" t="n">
         <v>4.97</v>
@@ -23753,7 +23753,7 @@
         <v>50.279</v>
       </c>
       <c r="C151" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D151" t="n">
         <v>5.002</v>
@@ -23781,7 +23781,7 @@
         <v>50.746</v>
       </c>
       <c r="C153" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D153" t="n">
         <v>5.094</v>
@@ -23823,7 +23823,7 @@
         <v>52.359</v>
       </c>
       <c r="C156" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D156" t="n">
         <v>5.368</v>
@@ -23837,7 +23837,7 @@
         <v>52.536</v>
       </c>
       <c r="C157" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D157" t="n">
         <v>5.401</v>
@@ -23851,7 +23851,7 @@
         <v>52.917</v>
       </c>
       <c r="C158" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D158" t="n">
         <v>5.477</v>
@@ -23879,7 +23879,7 @@
         <v>53.387</v>
       </c>
       <c r="C160" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D160" t="n">
         <v>5.561</v>
@@ -23893,7 +23893,7 @@
         <v>53.549</v>
       </c>
       <c r="C161" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D161" t="n">
         <v>5.593</v>
@@ -23935,7 +23935,7 @@
         <v>54.601</v>
       </c>
       <c r="C164" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D164" t="n">
         <v>5.774</v>
@@ -23963,7 +23963,7 @@
         <v>55.144</v>
       </c>
       <c r="C166" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D166" t="n">
         <v>5.874</v>
@@ -23991,7 +23991,7 @@
         <v>55.531</v>
       </c>
       <c r="C168" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D168" t="n">
         <v>5.952</v>
@@ -24033,7 +24033,7 @@
         <v>55.775</v>
       </c>
       <c r="C171" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D171" t="n">
         <v>6.005</v>
@@ -24075,7 +24075,7 @@
         <v>56.388</v>
       </c>
       <c r="C174" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D174" t="n">
         <v>6.146</v>
@@ -24103,7 +24103,7 @@
         <v>57.204</v>
       </c>
       <c r="C176" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D176" t="n">
         <v>6.344</v>
@@ -24145,7 +24145,7 @@
         <v>57.569</v>
       </c>
       <c r="C179" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D179" t="n">
         <v>6.437</v>
@@ -24159,7 +24159,7 @@
         <v>57.814</v>
       </c>
       <c r="C180" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D180" t="n">
         <v>6.494</v>
@@ -24215,7 +24215,7 @@
         <v>59.405</v>
       </c>
       <c r="C184" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D184" t="n">
         <v>6.829</v>
@@ -24271,7 +24271,7 @@
         <v>61.111</v>
       </c>
       <c r="C188" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D188" t="n">
         <v>7.141</v>
@@ -24467,7 +24467,7 @@
         <v>66.123</v>
       </c>
       <c r="C202" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D202" t="n">
         <v>7.888</v>
@@ -24495,7 +24495,7 @@
         <v>66.94499999999999</v>
       </c>
       <c r="C204" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D204" t="n">
         <v>7.988</v>
@@ -24523,7 +24523,7 @@
         <v>67.884</v>
       </c>
       <c r="C206" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D206" t="n">
         <v>8.085000000000001</v>
@@ -24565,7 +24565,7 @@
         <v>68.84</v>
       </c>
       <c r="C209" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D209" t="n">
         <v>8.167</v>
@@ -24579,7 +24579,7 @@
         <v>69.268</v>
       </c>
       <c r="C210" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D210" t="n">
         <v>8.196999999999999</v>
@@ -24635,7 +24635,7 @@
         <v>71.199</v>
       </c>
       <c r="C214" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D214" t="n">
         <v>8.300000000000001</v>
@@ -24663,7 +24663,7 @@
         <v>71.458</v>
       </c>
       <c r="C216" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D216" t="n">
         <v>8.317</v>
@@ -24677,7 +24677,7 @@
         <v>71.685</v>
       </c>
       <c r="C217" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D217" t="n">
         <v>8.329000000000001</v>
@@ -24733,7 +24733,7 @@
         <v>73.04300000000001</v>
       </c>
       <c r="C221" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D221" t="n">
         <v>8.378</v>
@@ -24761,7 +24761,7 @@
         <v>73.486</v>
       </c>
       <c r="C223" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D223" t="n">
         <v>8.388</v>
@@ -24775,7 +24775,7 @@
         <v>73.82599999999999</v>
       </c>
       <c r="C224" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D224" t="n">
         <v>8.391</v>
@@ -24817,7 +24817,7 @@
         <v>74.93899999999999</v>
       </c>
       <c r="C227" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D227" t="n">
         <v>8.385</v>
@@ -24831,7 +24831,7 @@
         <v>75.134</v>
       </c>
       <c r="C228" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D228" t="n">
         <v>8.381</v>
@@ -24845,7 +24845,7 @@
         <v>75.84099999999999</v>
       </c>
       <c r="C229" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D229" t="n">
         <v>8.359</v>
@@ -24859,7 +24859,7 @@
         <v>76.806</v>
       </c>
       <c r="C230" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D230" t="n">
         <v>8.317</v>
@@ -24873,7 +24873,7 @@
         <v>76.884</v>
       </c>
       <c r="C231" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D231" t="n">
         <v>8.313000000000001</v>
@@ -24887,7 +24887,7 @@
         <v>77.11799999999999</v>
       </c>
       <c r="C232" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D232" t="n">
         <v>8.297000000000001</v>
@@ -24915,7 +24915,7 @@
         <v>77.878</v>
       </c>
       <c r="C234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>8.234999999999999</v>
@@ -24943,7 +24943,7 @@
         <v>77.98</v>
       </c>
       <c r="C236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D236" t="n">
         <v>8.226000000000001</v>

</xml_diff>